<commit_message>
PreisWerk: Seiten-Aequivalente je Format hinterlegbar
Neue Spalte L "Seiten-Aequivalent" im Blatt "Preise" der Angebotsdaten.xlsx.
Ist dort eine Zahl eingetragen, gilt sie fuer das Format dieser Zeile; bleibt
die Zelle leer, wird der Wert wie bisher aus dem Formatnamen abgeleitet.

Die Ableitung liest jetzt einen Bruch im Namen als Bruch, statt auf einzelne
Textbausteine zu pruefen. Damit zaehlt "2/10 Seite" nicht mehr wie eine
Doppelseite (2,0), sondern als 0,2; ebenso richtig werden 2/3, 2/5 und 3/5.
Von 166 Formatnamen der Preisliste aendern sich genau diese acht, die uebrigen
158 bleiben unveraendert.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Angebotsdaten.xlsx
+++ b/Angebotsdaten.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11134" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11135" uniqueCount="704">
   <si>
     <t>Wird in der Vorlage über »Daten laden« eingelesen. Der Dateiname ist frei wählbar;</t>
   </si>
@@ -2308,6 +2308,9 @@
   <si>
     <t>Gehirn
 CME: Übergewicht und Adipositas im Kindes- und Jugendalter</t>
+  </si>
+  <si>
+    <t>Seiten-Äquivalent</t>
   </si>
 </sst>
 </file>
@@ -2901,7 +2904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K1449"/>
+  <dimension ref="A1:L1449"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="16" customWidth="1"/>
@@ -2915,9 +2918,10 @@
     <col min="9" max="9" width="10.85546875" style="16" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16" style="22" customWidth="1"/>
     <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>8</v>
       </c>
@@ -2950,6 +2954,9 @@
       </c>
       <c r="K1" s="3" t="s">
         <v>673</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Preisliste aus einer Datenbank, Excel bleibt Notweg
Alle vier Werkzeuge und die Startseite holen Preise und Termine zuerst aus
einer Supabase-Datenbank. Antwortet sie nicht, wird wie bisher die
Angebotsdaten.xlsx daneben gelesen; danach bleibt der Zwischenspeicher.
Die Statuszeile nennt die Herkunft.

Gelesen wird ohne Anmeldung, geaendert werden darf nur mit Freigabe.

Nachgewiesen: je Werkzeug beide Wege gegeneinander verglichen, Schluessel
fuer Schluessel und in der Reihenfolge. Abweichungen nur dort, wo bewusst
berichtigt wurde.

Dabei berichtigt:
- Anzeigenschluss Die Urologie 2027 Heft 1 verlor bisher seine Jahreszahl
  und erschien als 22.12.2027 bzw. als vollstaendige Datums-Zeichenkette.
- Werbebeilage bis 25g stand bei Die Kardiologie 2026 doppelt in der
  Auswahl von OpenSlots.
- Rechenrest 7920.000000000001 -> 7920.
- Termine mit eigener Jahreszahl jetzt ausgeschrieben (URO-NEWS 2026 Heft 1,
  Die Urologie 2027 Heft 1).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Angebotsdaten.xlsx
+++ b/Angebotsdaten.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11135" uniqueCount="704">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11136" uniqueCount="705">
   <si>
     <t>Wird in der Vorlage über »Daten laden« eingelesen. Der Dateiname ist frei wählbar;</t>
   </si>
@@ -1949,13 +1949,13 @@
     <t>19.10.</t>
   </si>
   <si>
-    <t>04.12.25</t>
-  </si>
-  <si>
-    <t>08.12.25</t>
-  </si>
-  <si>
-    <t>17.12.25</t>
+    <t>04.12.2025</t>
+  </si>
+  <si>
+    <t>08.12.2025</t>
+  </si>
+  <si>
+    <t>17.12.2025</t>
   </si>
   <si>
     <t>11.02.</t>
@@ -2311,6 +2311,9 @@
   </si>
   <si>
     <t>Seiten-Äquivalent</t>
+  </si>
+  <si>
+    <t>22.12.2026</t>
   </si>
 </sst>
 </file>
@@ -52394,8 +52397,8 @@
       <c r="E211" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="F211" s="21">
-        <v>46378</v>
+      <c r="F211" s="21" t="s">
+        <v>704</v>
       </c>
       <c r="G211" s="21" t="s">
         <v>468</v>

</xml_diff>

<commit_message>
Preisliste: Notweg auf den Stand der Datenbank gebracht
</commit_message>
<xml_diff>
--- a/Angebotsdaten.xlsx
+++ b/Angebotsdaten.xlsx
@@ -70844,7 +70844,10 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>DGP Kongress (Auslage), 03.03.–06.03.2027, Köln</t>
+          <t>DGP Kongress (Auslage), 03.03.–06.03.2027, Köln
+23. AIO-Herbstkongress 2026 (Bericht)
+68th ASH Annual Meeting and Exposition 2026 (ASH 2026) (Bericht)
+48th Annual San Antonio Breast Cancer Symposium (SABCS 2026)</t>
         </is>
       </c>
     </row>
@@ -71304,7 +71307,10 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>DGP Kongress (Auslage), 03.03.–06.03.2027, Köln</t>
+          <t>DGP Kongress (Auslage), 03.03.–06.03.2027, Köln
+23. AIO-Herbstkongress 2026 (Bericht)
+68th ASH Annual Meeting and Exposition 2026 (ASH 2026) (Bericht)
+48th Annual San Antonio Breast Cancer Symposium (SABCS 2026)</t>
         </is>
       </c>
     </row>
@@ -71570,7 +71576,9 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>DGP Kongress (Auslage), 03.03.–06.03.2027, Köln</t>
+          <t>DGP Kongress (Auslage), 03.03.–06.03.2027, Köln
+68th ASH Annual Meeting and Exposition 2026 (ASH 2026) (Bericht)
+48th Annual San Antonio Breast Cancer Symposium (SABCS 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>